<commit_message>
Sincroniza con el motor privado
</commit_message>
<xml_diff>
--- a/salida/cierre_3101789456_2026-03.xlsx
+++ b/salida/cierre_3101789456_2026-03.xlsx
@@ -12,7 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diario" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Balance comprobacion" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Excepciones" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F150 2026-03" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conciliacion XML" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F150 2026-03" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -27545,6 +27546,4660 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:J89"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>comprobante</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>contraparte</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>base_xml</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>base_registrada</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>iva_xml</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>iva_registrado</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>total_xml</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>total_registrado</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>diferencia</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>estado</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>00100001010000000001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Distribuidora Harinas del Valle S.A.</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>18400.00</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>18400.00</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2392.00</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>2392.00</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>20792.00</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>20792.00</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>00100001010000000002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Distribuidora Harinas del Valle S.A.</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>37500.00</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>37500.00</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>4875.00</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>4875.00</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>42375.00</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>42375.00</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>00100001010000000003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Compania Nacional de Fuerza y Luz</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>50000.00</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>50000.00</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>6500.00</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>6500.00</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>56500.00</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>56500.00</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>00100001010000000004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Compania Nacional de Fuerza y Luz</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>50000.00</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>50000.00</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>6500.00</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>6500.00</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>56500.00</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>56500.00</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>00100001010000000005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Compania Nacional de Fuerza y Luz</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>25000.00</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>25000.00</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>3250.00</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>3250.00</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>28250.00</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>28250.00</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>00100001010000000006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Servicentro El Roble S.A.</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>25000.00</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>25000.00</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>3250.00</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>3250.00</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>28250.00</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>28250.00</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>00100001010000000007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Servicentro El Roble S.A.</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>30600.00</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>30600.00</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>3978.00</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>3978.00</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>34578.00</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>34578.00</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>00100001010000000008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Servicentro El Roble S.A.</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>750000.00</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>750000.00</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>97500.00</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>97500.00</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>847500.00</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>847500.00</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>00100001010000000009</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Ana Rojas Vargas</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>36800.00</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>36800.00</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>4784.00</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>4784.00</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>41584.00</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>41584.00</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>00100001010000000010</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Inmobiliaria Perez Zeledon S.A.</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>250000.00</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>250000.00</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>32500.00</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>32500.00</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>282500.00</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>282500.00</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>00100001010000000011</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Seguros del Istmo Ltda.</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>273600.00</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>273600.00</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>5472.00</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>5472.00</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>279072.00</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>279072.00</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>00100001010000000012</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Seguros del Istmo Ltda.</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>22950.00</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>22950.00</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>459.00</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>459.00</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>23409.00</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>23409.00</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>00100001010000000013</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Suministros de Oficina CR S.A.</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>37500.00</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>37500.00</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>4875.00</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>4875.00</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>42375.00</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>42375.00</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>00100001010000000014</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Refrigeracion Tecnica del Sur S.A.</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>7650.00</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>7650.00</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>994.50</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>994.50</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>8644.50</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>8644.50</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>00100001010000000015</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Refrigeracion Tecnica del Sur S.A.</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>104400.00</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>104400.00</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>13572.00</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>13572.00</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>117972.00</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>117972.00</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>00100001010000000016</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Transportes Rapidos Zeledon S.A.</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>18400.00</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>18400.00</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>2392.00</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>2392.00</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>20792.00</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>20792.00</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>00100001010000000017</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Transportes Rapidos Zeledon S.A.</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>1000000.00</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>1000000.00</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>130000.00</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>130000.00</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>1130000.00</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>1130000.00</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>00100001010000000018</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Caja Costarricense de Seguro Social</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>30600.00</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>30600.00</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>30600.00</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>30600.00</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>00100001010000000019</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Comercial Zeta del Sur S.A.</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>73600.00</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>73600.00</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>9568.00</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>9568.00</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>83168.00</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>83168.00</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>00100001010000000020</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Servicios Integrales GYS S.A.</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>50000.00</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>50000.00</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>6500.00</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>6500.00</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>56500.00</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>56500.00</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>00100001010000000021</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Servicios Integrales GYS S.A.</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>50000.00</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>50000.00</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>6500.00</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>6500.00</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>56500.00</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>56500.00</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>00100001010000000022</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Servicios Integrales GYS S.A.</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>69600.00</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>69600.00</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>9048.00</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>9048.00</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>78648.00</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>78648.00</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>00100001010000000023</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Marvin Solis Mora</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>25000.00</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>25000.00</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>3250.00</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>3250.00</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>28250.00</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>28250.00</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>00100001010000000024</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Marvin Solis Mora</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>15300.00</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>15300.00</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>1989.00</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>1989.00</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>17289.00</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>17289.00</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>00100001010000000025</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Almacen El Progreso Ltda.</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>30600.00</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>30600.00</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>3978.00</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>3978.00</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>34578.00</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>34578.00</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>00100001010000000026</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Almacen El Progreso Ltda.</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>69600.00</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>69600.00</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>9048.00</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>9048.00</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>78648.00</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>78648.00</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>00100001010000000027</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Almacen El Progreso Ltda.</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>50000.00</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>50000.00</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>6500.00</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>6500.00</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>56500.00</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>56500.00</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>00100001030000000088</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Supermercado Central del Sur S.A.</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>13500.00</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>13500.00</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>135.00</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>135.00</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>13635.00</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>13635.00</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>00100001010000000028</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Supermercado Central del Sur S.A.</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>176400.00</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>176400.00</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>22932.00</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>22932.00</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>199332.00</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>199332.00</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>00100001010000000029</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Supermercado Central del Sur S.A.</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>446500.00</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>446500.00</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>42085.00</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>42085.00</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>488585.00</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>488585.00</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>00100001010000000030</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Supermercado Central del Sur S.A.</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>32400.00</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>32400.00</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>4212.00</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>4212.00</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>36612.00</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>36612.00</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>00100001010000000031</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Supermercado Central del Sur S.A.</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>75600.00</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>75600.00</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>756.00</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>756.00</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>76356.00</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>76356.00</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>00100001010000000032</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Supermercado Central del Sur S.A.</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>71400.00</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>71400.00</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>9282.00</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>9282.00</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>80682.00</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>80682.00</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>00100001010000000033</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Soda El Buen Sabor S.R.L.</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>370500.00</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>370500.00</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>3705.00</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>3705.00</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>374205.00</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>374205.00</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>00100001010000000034</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Supermercado Central del Sur S.A.</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>231000.00</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>231000.00</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>2310.00</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>2310.00</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>233310.00</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>233310.00</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>00100001040000000035</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Consumidor final</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>354000.00</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>354000.00</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>31764.00</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>31764.00</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>385764.00</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>385764.00</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>00100001040000000036</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Consumidor final</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>296400.00</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>296400.00</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>17364.00</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>17364.00</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>313764.00</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>313764.00</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>00100001010000000037</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Soda El Buen Sabor S.R.L.</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>251400.00</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>251400.00</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>21666.00</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>21666.00</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>273066.00</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>273066.00</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>00100001010000000038</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Hotel Montaña Verde S.A.</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>67500.00</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>67500.00</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>4575.00</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>4575.00</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>72075.00</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>72075.00</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>00100001040000000039</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Consumidor final</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>312000.00</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>312000.00</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>3120.00</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>3120.00</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>315120.00</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>315120.00</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>00100001040000000040</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Consumidor final</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>367100.00</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>367100.00</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>18491.00</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>18491.00</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>385591.00</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>385591.00</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>00100001010000000041</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Supermercado Central del Sur S.A.</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>597500.00</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>597500.00</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>23675.00</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>23675.00</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>621175.00</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>621175.00</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>00100001040000000042</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Consumidor final</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>296200.00</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>296200.00</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>13462.00</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>13462.00</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>309662.00</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>309662.00</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>00100001040000000043</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Consumidor final</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>516600.00</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>516600.00</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>53046.00</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>53046.00</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>569646.00</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>569646.00</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>00100001010000000044</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Hotel Montaña Verde S.A.</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>113800.00</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>113800.00</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>14794.00</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>14794.00</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>128594.00</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>128594.00</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>00100001010000000045</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Supermercado Central del Sur S.A.</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>161500.00</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>161500.00</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>1615.00</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>1615.00</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>163115.00</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>163115.00</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>00100001010000000046</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Hotel Montaña Verde S.A.</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>205100.00</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>205100.00</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>21263.00</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>21263.00</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>226363.00</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>226363.00</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>00100001010000000047</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Supermercado Central del Sur S.A.</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>318400.00</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>318400.00</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>41392.00</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>41392.00</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>359792.00</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>359792.00</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>00100001010000000048</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Soda El Buen Sabor S.R.L.</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>258700.00</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>258700.00</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>20731.00</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>20731.00</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>279431.00</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>279431.00</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>00100001010000000049</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Supermercado Central del Sur S.A.</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>335100.00</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>335100.00</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>15879.00</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>15879.00</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>350979.00</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>350979.00</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>00100001040000000050</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Consumidor final</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>230500.00</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>230500.00</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>14005.00</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>14005.00</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>244505.00</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>244505.00</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>00100001010000000051</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Soda El Buen Sabor S.R.L.</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>361200.00</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>361200.00</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>40908.00</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>40908.00</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>402108.00</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>402108.00</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>00100001010000000052</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Soda El Buen Sabor S.R.L.</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>193800.00</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>193800.00</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>1938.00</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>1938.00</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>195738.00</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>195738.00</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>00100001010000000053</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Supermercado Central del Sur S.A.</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>45000.00</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>45000.00</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>5850.00</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>5850.00</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>50850.00</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>50850.00</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>00100001010000000054</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Soda El Buen Sabor S.R.L.</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>672000.00</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>672000.00</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>54600.00</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>54600.00</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>726600.00</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>726600.00</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>00100001040000000055</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Consumidor final</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>264000.00</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>264000.00</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>2640.00</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>2640.00</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>266640.00</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>266640.00</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>00100001010000000056</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Supermercado Central del Sur S.A.</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>442100.00</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>442100.00</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>4421.00</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>4421.00</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>446521.00</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>446521.00</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>00100001010000000057</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Supermercado Central del Sur S.A.</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>204100.00</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>204100.00</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>15649.00</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>15649.00</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>219749.00</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>219749.00</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>00100001040000000058</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Consumidor final</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>57600.00</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>57600.00</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>5760.00</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>5760.00</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>63360.00</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>63360.00</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>00100001040000000059</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Consumidor final</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>1045000.00</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>1045000.00</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>67450.00</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>67450.00</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>1112450.00</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>1112450.00</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>00100001040000000060</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Consumidor final</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>50000.00</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>50000.00</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>6500.00</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>6500.00</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>56500.00</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>56500.00</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>00100001040000000061</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Consumidor final</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>201600.00</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>201600.00</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>2016.00</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>2016.00</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>203616.00</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>203616.00</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>00100001010000000062</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Supermercado Central del Sur S.A.</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>428400.00</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>428400.00</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>44292.00</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>44292.00</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>472692.00</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>472692.00</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>00100001010000000063</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Soda El Buen Sabor S.R.L.</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>130200.00</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>130200.00</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>16926.00</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>16926.00</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>147126.00</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>147126.00</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>00100001010000000064</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Hotel Montaña Verde S.A.</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>34200.00</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>34200.00</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>4446.00</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>4446.00</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>38646.00</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>38646.00</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>00100001010000000065</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Soda El Buen Sabor S.R.L.</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>126600.00</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>126600.00</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>1266.00</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>1266.00</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>127866.00</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>127866.00</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>00100001010000000066</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Supermercado Central del Sur S.A.</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>100000.00</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>100000.00</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>1000.00</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>1000.00</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>101000.00</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>101000.00</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>00100001010000000067</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Soda El Buen Sabor S.R.L.</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>135000.00</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>135000.00</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>17550.00</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>17550.00</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>152550.00</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>152550.00</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>00100001010000000068</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Soda El Buen Sabor S.R.L.</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>198400.00</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>198400.00</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>4792.00</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>4792.00</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>203192.00</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>203192.00</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>00100001010000000069</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Soda El Buen Sabor S.R.L.</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>359800.00</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>359800.00</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>32374.00</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>32374.00</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>392174.00</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>392174.00</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>00100001010000000070</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Supermercado Central del Sur S.A.</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>238200.00</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>238200.00</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>9582.00</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>9582.00</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>247782.00</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>247782.00</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>00100001010000000071</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Soda El Buen Sabor S.R.L.</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>262200.00</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>262200.00</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>21774.00</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>21774.00</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>283974.00</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>283974.00</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>00100001040000000072</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Consumidor final</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>348500.00</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>348500.00</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>45305.00</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>45305.00</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>393805.00</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>393805.00</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>00100001010000000073</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Soda El Buen Sabor S.R.L.</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>308700.00</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>308700.00</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>16191.00</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>16191.00</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>324891.00</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>324891.00</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>00100001010000000074</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Supermercado Central del Sur S.A.</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>429400.00</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>429400.00</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>33934.00</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>33934.00</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>463334.00</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>463334.00</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>00100001040000000075</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Consumidor final</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>71400.00</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>71400.00</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>714.00</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>714.00</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>72114.00</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>72114.00</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>00100001010000000076</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Hotel Montaña Verde S.A.</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>209000.00</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>209000.00</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>27170.00</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>27170.00</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>236170.00</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>236170.00</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>00100001040000000077</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Consumidor final</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>484500.00</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>484500.00</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>62985.00</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>62985.00</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>547485.00</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>547485.00</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>00100001040000000078</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Consumidor final</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>102600.00</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>102600.00</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>7074.00</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>7074.00</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>109674.00</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>109674.00</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>00100001010000000079</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Soda El Buen Sabor S.R.L.</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>95400.00</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>95400.00</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>954.00</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>954.00</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>96354.00</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>96354.00</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>00100001010000000080</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Supermercado Central del Sur S.A.</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>197400.00</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>197400.00</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>25662.00</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>25662.00</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>223062.00</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>223062.00</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>00100001010000000081</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Supermercado Central del Sur S.A.</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>327600.00</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>327600.00</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>32508.00</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>32508.00</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>360108.00</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>360108.00</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>00100001010000000082</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Soda El Buen Sabor S.R.L.</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>400300.00</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>400300.00</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>14803.00</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>14803.00</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>415103.00</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>415103.00</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>00100001040000000083</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Consumidor final</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>142800.00</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>142800.00</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>18564.00</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>18564.00</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>161364.00</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>161364.00</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>00100001010000000084</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Hotel Montaña Verde S.A.</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>398500.00</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>398500.00</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>8485.00</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>8485.00</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>406985.00</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>406985.00</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>00100001010000000085</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Soda El Buen Sabor S.R.L.</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>727000.00</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>727000.00</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>30670.00</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>30670.00</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>757670.00</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>757670.00</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>00100001010000000086</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Hotel Montaña Verde S.A.</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>363200.00</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>363200.00</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>13892.00</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>13892.00</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>377092.00</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>377092.00</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>00100001040000000087</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Consumidor final</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>264600.00</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>264600.00</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>14742.00</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>14742.00</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>279342.00</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>279342.00</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>